<commit_message>
Add the project number from the register
A ProjectNumber column in the project register (aliases ProjectNo,
JobNumber and the like, and listed under Match the register columns) is
now read with each project and shown:

- on the projects page, above each project's name, and searchable;
- in the project dashboard's header;
- on the cover sheet as a Project number field, filled from the
  register (tagged auto) and editable;
- on the letter, as a Project Number line directly under Project.

It is saved with the variation and sent to the log write as
projectNumber, for an optional ProjectNumber column. Optional: a project
without one shows nothing and is never reported as missing.

Docs: the register column, the Get projects Select line and the optional
log column. The register workbook and CSV gain the column.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0179JD8tKBuQw572uHNzHE2b
</commit_message>
<xml_diff>
--- a/registers/Variation Project Register.xlsx
+++ b/registers/Variation Project Register.xlsx
@@ -262,9 +262,9 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ProjectRegister" displayName="ProjectRegister" ref="A4:M8" headerRowCount="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ProjectRegister" displayName="ProjectRegister" ref="A4:N8" headerRowCount="1">
   <autoFilter ref="A4:M8"/>
-  <tableColumns count="13">
+  <tableColumns count="14">
     <tableColumn id="1" name="Title"/>
     <tableColumn id="2" name="State"/>
     <tableColumn id="3" name="HeadContractor"/>
@@ -278,6 +278,7 @@
     <tableColumn id="11" name="Active"/>
     <tableColumn id="12" name="PmEmail"/>
     <tableColumn id="13" name="RatesFile"/>
+    <tableColumn id="14" name="ProjectNumber"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight9" showRowStripes="1"/>
 </table>
@@ -572,7 +573,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M10"/>
+  <dimension ref="A1:N10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -588,6 +589,7 @@
     <col width="9" customWidth="1" min="11" max="11"/>
     <col width="34" customWidth="1" min="12" max="12"/>
     <col width="48" customWidth="1" min="13" max="13"/>
+    <col width="16" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
@@ -670,6 +672,11 @@
           <t>RatesFile</t>
         </is>
       </c>
+      <c r="N4" s="3" t="inlineStr">
+        <is>
+          <t>ProjectNumber</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="44" customHeight="1">
       <c r="A5" s="4" t="inlineStr">
@@ -734,6 +741,11 @@
           <t>/Shared Documents/25-135 Warrnambool Hospital/Agreed Schedule of Rates.xlsx</t>
         </is>
       </c>
+      <c r="N5" s="4" t="inlineStr">
+        <is>
+          <t>25-135</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="44" customHeight="1">
       <c r="A6" s="4" t="inlineStr">
@@ -791,6 +803,11 @@
         </is>
       </c>
       <c r="M6" s="4" t="n"/>
+      <c r="N6" s="4" t="inlineStr">
+        <is>
+          <t>24-902</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="44" customHeight="1">
       <c r="A7" s="4" t="inlineStr">
@@ -847,6 +864,11 @@
         </is>
       </c>
       <c r="M7" s="4" t="n"/>
+      <c r="N7" s="4" t="inlineStr">
+        <is>
+          <t>25-018</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="44" customHeight="1">
       <c r="A8" s="4" t="inlineStr">
@@ -895,8 +917,12 @@
       </c>
       <c r="L8" s="4" t="inlineStr"/>
       <c r="M8" s="4" t="n"/>
+      <c r="N8" s="4" t="inlineStr">
+        <is>
+          <t>25-204</t>
+        </is>
+      </c>
     </row>
-    <row r="9"/>
     <row r="10">
       <c r="A10" s="6" t="inlineStr">
         <is>

</xml_diff>